<commit_message>
New Monitoring Dashboard, Multiple Updates - Major Update 2
</commit_message>
<xml_diff>
--- a/backend/onboarding/templates/1_Schools_And_Chairmen.xlsx
+++ b/backend/onboarding/templates/1_Schools_And_Chairmen.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>IECE — SCHOOL &amp; CHAIRMAN ONBOARDING SHEET</t>
   </si>
@@ -83,10 +83,6 @@
   <si>
     <t xml:space="preserve">Class Coverage
 (e.g. 8th to 10th)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Strength
-(optional — e.g. 450)</t>
   </si>
 </sst>
 </file>
@@ -543,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -553,10 +549,9 @@
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -566,9 +561,8 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -578,9 +572,8 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" ht="46" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" ht="46" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -602,11 +595,8 @@
       <c r="G3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="6"/>
@@ -614,9 +604,8 @@
       <c r="E4" s="5"/>
       <c r="F4" s="7"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="6"/>
@@ -624,9 +613,8 @@
       <c r="E5" s="5"/>
       <c r="F5" s="7"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="6"/>
@@ -634,9 +622,8 @@
       <c r="E6" s="5"/>
       <c r="F6" s="7"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="6"/>
@@ -644,9 +631,8 @@
       <c r="E7" s="5"/>
       <c r="F7" s="7"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="6"/>
@@ -654,9 +640,8 @@
       <c r="E8" s="5"/>
       <c r="F8" s="7"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="6"/>
@@ -664,9 +649,8 @@
       <c r="E9" s="5"/>
       <c r="F9" s="7"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -674,9 +658,8 @@
       <c r="E10" s="5"/>
       <c r="F10" s="7"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -684,9 +667,8 @@
       <c r="E11" s="5"/>
       <c r="F11" s="7"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -694,9 +676,8 @@
       <c r="E12" s="5"/>
       <c r="F12" s="7"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -704,9 +685,8 @@
       <c r="E13" s="5"/>
       <c r="F13" s="7"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -714,9 +694,8 @@
       <c r="E14" s="5"/>
       <c r="F14" s="7"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="6"/>
@@ -724,9 +703,8 @@
       <c r="E15" s="5"/>
       <c r="F15" s="7"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="6"/>
@@ -734,9 +712,8 @@
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="6"/>
@@ -744,9 +721,8 @@
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="6"/>
@@ -754,9 +730,8 @@
       <c r="E18" s="5"/>
       <c r="F18" s="7"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="6"/>
@@ -764,9 +739,8 @@
       <c r="E19" s="5"/>
       <c r="F19" s="7"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="6"/>
@@ -774,9 +748,8 @@
       <c r="E20" s="5"/>
       <c r="F20" s="7"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="6"/>
@@ -784,9 +757,8 @@
       <c r="E21" s="5"/>
       <c r="F21" s="7"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="6"/>
@@ -794,9 +766,8 @@
       <c r="E22" s="5"/>
       <c r="F22" s="7"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="6"/>
@@ -804,9 +775,8 @@
       <c r="E23" s="5"/>
       <c r="F23" s="7"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="6"/>
@@ -814,9 +784,8 @@
       <c r="E24" s="5"/>
       <c r="F24" s="7"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="6"/>
@@ -824,9 +793,8 @@
       <c r="E25" s="5"/>
       <c r="F25" s="7"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="6"/>
@@ -834,9 +802,8 @@
       <c r="E26" s="5"/>
       <c r="F26" s="7"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
@@ -844,9 +811,8 @@
       <c r="E27" s="5"/>
       <c r="F27" s="7"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="6"/>
@@ -854,9 +820,8 @@
       <c r="E28" s="5"/>
       <c r="F28" s="7"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="6"/>
@@ -864,9 +829,8 @@
       <c r="E29" s="5"/>
       <c r="F29" s="7"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="6"/>
@@ -874,9 +838,8 @@
       <c r="E30" s="5"/>
       <c r="F30" s="7"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="6"/>
@@ -884,9 +847,8 @@
       <c r="E31" s="5"/>
       <c r="F31" s="7"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="6"/>
@@ -894,9 +856,8 @@
       <c r="E32" s="5"/>
       <c r="F32" s="7"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="6"/>
@@ -904,9 +865,8 @@
       <c r="E33" s="5"/>
       <c r="F33" s="7"/>
       <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="6"/>
@@ -914,9 +874,8 @@
       <c r="E34" s="5"/>
       <c r="F34" s="7"/>
       <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="6"/>
@@ -924,9 +883,8 @@
       <c r="E35" s="5"/>
       <c r="F35" s="7"/>
       <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="6"/>
@@ -934,9 +892,8 @@
       <c r="E36" s="5"/>
       <c r="F36" s="7"/>
       <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="6"/>
@@ -944,9 +901,8 @@
       <c r="E37" s="5"/>
       <c r="F37" s="7"/>
       <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="6"/>
@@ -954,9 +910,8 @@
       <c r="E38" s="5"/>
       <c r="F38" s="7"/>
       <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="6"/>
@@ -964,9 +919,8 @@
       <c r="E39" s="5"/>
       <c r="F39" s="7"/>
       <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
       <c r="B40" s="5"/>
       <c r="C40" s="6"/>
@@ -974,9 +928,8 @@
       <c r="E40" s="5"/>
       <c r="F40" s="7"/>
       <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
       <c r="B41" s="5"/>
       <c r="C41" s="6"/>
@@ -984,9 +937,8 @@
       <c r="E41" s="5"/>
       <c r="F41" s="7"/>
       <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="6"/>
@@ -994,9 +946,8 @@
       <c r="E42" s="5"/>
       <c r="F42" s="7"/>
       <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
       <c r="B43" s="5"/>
       <c r="C43" s="6"/>
@@ -1004,9 +955,8 @@
       <c r="E43" s="5"/>
       <c r="F43" s="7"/>
       <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
       <c r="B44" s="5"/>
       <c r="C44" s="6"/>
@@ -1014,9 +964,8 @@
       <c r="E44" s="5"/>
       <c r="F44" s="7"/>
       <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="5"/>
       <c r="B45" s="5"/>
       <c r="C45" s="6"/>
@@ -1024,9 +973,8 @@
       <c r="E45" s="5"/>
       <c r="F45" s="7"/>
       <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="5"/>
       <c r="B46" s="5"/>
       <c r="C46" s="6"/>
@@ -1034,9 +982,8 @@
       <c r="E46" s="5"/>
       <c r="F46" s="7"/>
       <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
       <c r="B47" s="5"/>
       <c r="C47" s="6"/>
@@ -1044,9 +991,8 @@
       <c r="E47" s="5"/>
       <c r="F47" s="7"/>
       <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
       <c r="B48" s="5"/>
       <c r="C48" s="6"/>
@@ -1054,9 +1000,8 @@
       <c r="E48" s="5"/>
       <c r="F48" s="7"/>
       <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="5"/>
       <c r="B49" s="5"/>
       <c r="C49" s="6"/>
@@ -1064,9 +1009,8 @@
       <c r="E49" s="5"/>
       <c r="F49" s="7"/>
       <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
       <c r="B50" s="5"/>
       <c r="C50" s="6"/>
@@ -1074,9 +1018,8 @@
       <c r="E50" s="5"/>
       <c r="F50" s="7"/>
       <c r="G50" s="5"/>
-      <c r="H50" s="5"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
       <c r="B51" s="5"/>
       <c r="C51" s="6"/>
@@ -1084,9 +1027,8 @@
       <c r="E51" s="5"/>
       <c r="F51" s="7"/>
       <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
       <c r="B52" s="5"/>
       <c r="C52" s="6"/>
@@ -1094,9 +1036,8 @@
       <c r="E52" s="5"/>
       <c r="F52" s="7"/>
       <c r="G52" s="5"/>
-      <c r="H52" s="5"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="5"/>
       <c r="B53" s="5"/>
       <c r="C53" s="6"/>
@@ -1104,9 +1045,8 @@
       <c r="E53" s="5"/>
       <c r="F53" s="7"/>
       <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="5"/>
       <c r="B54" s="5"/>
       <c r="C54" s="6"/>
@@ -1114,9 +1054,8 @@
       <c r="E54" s="5"/>
       <c r="F54" s="7"/>
       <c r="G54" s="5"/>
-      <c r="H54" s="5"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="5"/>
       <c r="B55" s="5"/>
       <c r="C55" s="6"/>
@@ -1124,9 +1063,8 @@
       <c r="E55" s="5"/>
       <c r="F55" s="7"/>
       <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="C56" s="6"/>
@@ -1134,9 +1072,8 @@
       <c r="E56" s="5"/>
       <c r="F56" s="7"/>
       <c r="G56" s="5"/>
-      <c r="H56" s="5"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="6"/>
@@ -1144,9 +1081,8 @@
       <c r="E57" s="5"/>
       <c r="F57" s="7"/>
       <c r="G57" s="5"/>
-      <c r="H57" s="5"/>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="5"/>
       <c r="B58" s="5"/>
       <c r="C58" s="6"/>
@@ -1154,9 +1090,8 @@
       <c r="E58" s="5"/>
       <c r="F58" s="7"/>
       <c r="G58" s="5"/>
-      <c r="H58" s="5"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="5"/>
       <c r="B59" s="5"/>
       <c r="C59" s="6"/>
@@ -1164,9 +1099,8 @@
       <c r="E59" s="5"/>
       <c r="F59" s="7"/>
       <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="5"/>
       <c r="B60" s="5"/>
       <c r="C60" s="6"/>
@@ -1174,9 +1108,8 @@
       <c r="E60" s="5"/>
       <c r="F60" s="7"/>
       <c r="G60" s="5"/>
-      <c r="H60" s="5"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="5"/>
       <c r="B61" s="5"/>
       <c r="C61" s="6"/>
@@ -1184,9 +1117,8 @@
       <c r="E61" s="5"/>
       <c r="F61" s="7"/>
       <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="5"/>
       <c r="B62" s="5"/>
       <c r="C62" s="6"/>
@@ -1194,9 +1126,8 @@
       <c r="E62" s="5"/>
       <c r="F62" s="7"/>
       <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="5"/>
       <c r="B63" s="5"/>
       <c r="C63" s="6"/>
@@ -1204,9 +1135,8 @@
       <c r="E63" s="5"/>
       <c r="F63" s="7"/>
       <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="6"/>
@@ -1214,9 +1144,8 @@
       <c r="E64" s="5"/>
       <c r="F64" s="7"/>
       <c r="G64" s="5"/>
-      <c r="H64" s="5"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="5"/>
       <c r="B65" s="5"/>
       <c r="C65" s="6"/>
@@ -1224,9 +1153,8 @@
       <c r="E65" s="5"/>
       <c r="F65" s="7"/>
       <c r="G65" s="5"/>
-      <c r="H65" s="5"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="5"/>
       <c r="B66" s="5"/>
       <c r="C66" s="6"/>
@@ -1234,9 +1162,8 @@
       <c r="E66" s="5"/>
       <c r="F66" s="7"/>
       <c r="G66" s="5"/>
-      <c r="H66" s="5"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
       <c r="C67" s="6"/>
@@ -1244,9 +1171,8 @@
       <c r="E67" s="5"/>
       <c r="F67" s="7"/>
       <c r="G67" s="5"/>
-      <c r="H67" s="5"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="5"/>
       <c r="B68" s="5"/>
       <c r="C68" s="6"/>
@@ -1254,9 +1180,8 @@
       <c r="E68" s="5"/>
       <c r="F68" s="7"/>
       <c r="G68" s="5"/>
-      <c r="H68" s="5"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="5"/>
       <c r="B69" s="5"/>
       <c r="C69" s="6"/>
@@ -1264,9 +1189,8 @@
       <c r="E69" s="5"/>
       <c r="F69" s="7"/>
       <c r="G69" s="5"/>
-      <c r="H69" s="5"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="5"/>
       <c r="B70" s="5"/>
       <c r="C70" s="6"/>
@@ -1274,9 +1198,8 @@
       <c r="E70" s="5"/>
       <c r="F70" s="7"/>
       <c r="G70" s="5"/>
-      <c r="H70" s="5"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="5"/>
       <c r="B71" s="5"/>
       <c r="C71" s="6"/>
@@ -1284,9 +1207,8 @@
       <c r="E71" s="5"/>
       <c r="F71" s="7"/>
       <c r="G71" s="5"/>
-      <c r="H71" s="5"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="5"/>
       <c r="B72" s="5"/>
       <c r="C72" s="6"/>
@@ -1294,9 +1216,8 @@
       <c r="E72" s="5"/>
       <c r="F72" s="7"/>
       <c r="G72" s="5"/>
-      <c r="H72" s="5"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="5"/>
       <c r="B73" s="5"/>
       <c r="C73" s="6"/>
@@ -1304,9 +1225,8 @@
       <c r="E73" s="5"/>
       <c r="F73" s="7"/>
       <c r="G73" s="5"/>
-      <c r="H73" s="5"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="5"/>
       <c r="B74" s="5"/>
       <c r="C74" s="6"/>
@@ -1314,9 +1234,8 @@
       <c r="E74" s="5"/>
       <c r="F74" s="7"/>
       <c r="G74" s="5"/>
-      <c r="H74" s="5"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="5"/>
       <c r="B75" s="5"/>
       <c r="C75" s="6"/>
@@ -1324,9 +1243,8 @@
       <c r="E75" s="5"/>
       <c r="F75" s="7"/>
       <c r="G75" s="5"/>
-      <c r="H75" s="5"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="5"/>
       <c r="B76" s="5"/>
       <c r="C76" s="6"/>
@@ -1334,9 +1252,8 @@
       <c r="E76" s="5"/>
       <c r="F76" s="7"/>
       <c r="G76" s="5"/>
-      <c r="H76" s="5"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="C77" s="6"/>
@@ -1344,9 +1261,8 @@
       <c r="E77" s="5"/>
       <c r="F77" s="7"/>
       <c r="G77" s="5"/>
-      <c r="H77" s="5"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="5"/>
       <c r="B78" s="5"/>
       <c r="C78" s="6"/>
@@ -1354,9 +1270,8 @@
       <c r="E78" s="5"/>
       <c r="F78" s="7"/>
       <c r="G78" s="5"/>
-      <c r="H78" s="5"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="5"/>
       <c r="B79" s="5"/>
       <c r="C79" s="6"/>
@@ -1364,9 +1279,8 @@
       <c r="E79" s="5"/>
       <c r="F79" s="7"/>
       <c r="G79" s="5"/>
-      <c r="H79" s="5"/>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="5"/>
       <c r="B80" s="5"/>
       <c r="C80" s="6"/>
@@ -1374,9 +1288,8 @@
       <c r="E80" s="5"/>
       <c r="F80" s="7"/>
       <c r="G80" s="5"/>
-      <c r="H80" s="5"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="6"/>
@@ -1384,9 +1297,8 @@
       <c r="E81" s="5"/>
       <c r="F81" s="7"/>
       <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
       <c r="C82" s="6"/>
@@ -1394,9 +1306,8 @@
       <c r="E82" s="5"/>
       <c r="F82" s="7"/>
       <c r="G82" s="5"/>
-      <c r="H82" s="5"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="5"/>
       <c r="B83" s="5"/>
       <c r="C83" s="6"/>
@@ -1404,9 +1315,8 @@
       <c r="E83" s="5"/>
       <c r="F83" s="7"/>
       <c r="G83" s="5"/>
-      <c r="H83" s="5"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="5"/>
       <c r="B84" s="5"/>
       <c r="C84" s="6"/>
@@ -1414,9 +1324,8 @@
       <c r="E84" s="5"/>
       <c r="F84" s="7"/>
       <c r="G84" s="5"/>
-      <c r="H84" s="5"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="5"/>
       <c r="B85" s="5"/>
       <c r="C85" s="6"/>
@@ -1424,9 +1333,8 @@
       <c r="E85" s="5"/>
       <c r="F85" s="7"/>
       <c r="G85" s="5"/>
-      <c r="H85" s="5"/>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="5"/>
       <c r="B86" s="5"/>
       <c r="C86" s="6"/>
@@ -1434,9 +1342,8 @@
       <c r="E86" s="5"/>
       <c r="F86" s="7"/>
       <c r="G86" s="5"/>
-      <c r="H86" s="5"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="5"/>
       <c r="B87" s="5"/>
       <c r="C87" s="6"/>
@@ -1444,9 +1351,8 @@
       <c r="E87" s="5"/>
       <c r="F87" s="7"/>
       <c r="G87" s="5"/>
-      <c r="H87" s="5"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="5"/>
       <c r="B88" s="5"/>
       <c r="C88" s="6"/>
@@ -1454,9 +1360,8 @@
       <c r="E88" s="5"/>
       <c r="F88" s="7"/>
       <c r="G88" s="5"/>
-      <c r="H88" s="5"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="5"/>
       <c r="B89" s="5"/>
       <c r="C89" s="6"/>
@@ -1464,9 +1369,8 @@
       <c r="E89" s="5"/>
       <c r="F89" s="7"/>
       <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="5"/>
       <c r="B90" s="5"/>
       <c r="C90" s="6"/>
@@ -1474,9 +1378,8 @@
       <c r="E90" s="5"/>
       <c r="F90" s="7"/>
       <c r="G90" s="5"/>
-      <c r="H90" s="5"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="5"/>
       <c r="B91" s="5"/>
       <c r="C91" s="6"/>
@@ -1484,9 +1387,8 @@
       <c r="E91" s="5"/>
       <c r="F91" s="7"/>
       <c r="G91" s="5"/>
-      <c r="H91" s="5"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="5"/>
       <c r="B92" s="5"/>
       <c r="C92" s="6"/>
@@ -1494,9 +1396,8 @@
       <c r="E92" s="5"/>
       <c r="F92" s="7"/>
       <c r="G92" s="5"/>
-      <c r="H92" s="5"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="5"/>
       <c r="B93" s="5"/>
       <c r="C93" s="6"/>
@@ -1504,9 +1405,8 @@
       <c r="E93" s="5"/>
       <c r="F93" s="7"/>
       <c r="G93" s="5"/>
-      <c r="H93" s="5"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="5"/>
       <c r="B94" s="5"/>
       <c r="C94" s="6"/>
@@ -1514,9 +1414,8 @@
       <c r="E94" s="5"/>
       <c r="F94" s="7"/>
       <c r="G94" s="5"/>
-      <c r="H94" s="5"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="5"/>
       <c r="B95" s="5"/>
       <c r="C95" s="6"/>
@@ -1524,9 +1423,8 @@
       <c r="E95" s="5"/>
       <c r="F95" s="7"/>
       <c r="G95" s="5"/>
-      <c r="H95" s="5"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="5"/>
       <c r="B96" s="5"/>
       <c r="C96" s="6"/>
@@ -1534,9 +1432,8 @@
       <c r="E96" s="5"/>
       <c r="F96" s="7"/>
       <c r="G96" s="5"/>
-      <c r="H96" s="5"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="5"/>
       <c r="B97" s="5"/>
       <c r="C97" s="6"/>
@@ -1544,9 +1441,8 @@
       <c r="E97" s="5"/>
       <c r="F97" s="7"/>
       <c r="G97" s="5"/>
-      <c r="H97" s="5"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="5"/>
       <c r="B98" s="5"/>
       <c r="C98" s="6"/>
@@ -1554,9 +1450,8 @@
       <c r="E98" s="5"/>
       <c r="F98" s="7"/>
       <c r="G98" s="5"/>
-      <c r="H98" s="5"/>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="5"/>
       <c r="B99" s="5"/>
       <c r="C99" s="6"/>
@@ -1564,9 +1459,8 @@
       <c r="E99" s="5"/>
       <c r="F99" s="7"/>
       <c r="G99" s="5"/>
-      <c r="H99" s="5"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="5"/>
       <c r="B100" s="5"/>
       <c r="C100" s="6"/>
@@ -1574,9 +1468,8 @@
       <c r="E100" s="5"/>
       <c r="F100" s="7"/>
       <c r="G100" s="5"/>
-      <c r="H100" s="5"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="5"/>
       <c r="B101" s="5"/>
       <c r="C101" s="6"/>
@@ -1584,9 +1477,8 @@
       <c r="E101" s="5"/>
       <c r="F101" s="7"/>
       <c r="G101" s="5"/>
-      <c r="H101" s="5"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="5"/>
       <c r="B102" s="5"/>
       <c r="C102" s="6"/>
@@ -1594,9 +1486,8 @@
       <c r="E102" s="5"/>
       <c r="F102" s="7"/>
       <c r="G102" s="5"/>
-      <c r="H102" s="5"/>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="5"/>
       <c r="B103" s="5"/>
       <c r="C103" s="6"/>
@@ -1604,13 +1495,12 @@
       <c r="E103" s="5"/>
       <c r="F103" s="7"/>
       <c r="G103" s="5"/>
-      <c r="H103" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H3"/>
+  <autoFilter ref="A3:G3"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>